<commit_message>
descargados e incluidos todos los archivos enviados en emails del departamento de mates (examenes, materiales, etc)
</commit_message>
<xml_diff>
--- a/hipoteca/tabla_amortizaciones.xlsx
+++ b/hipoteca/tabla_amortizaciones.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ac4744725179635e/Desktop/sapere_aude/hipoteca/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="79" documentId="13_ncr:1_{6A36A00E-2702-4A70-A591-6BDDD99505EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{535C6F4C-DE33-4204-AB34-E0B7590838D5}"/>
+  <xr:revisionPtr revIDLastSave="96" documentId="13_ncr:1_{6A36A00E-2702-4A70-A591-6BDDD99505EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B3DD07E-2304-4F05-A681-AFDE568B93F7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="29">
   <si>
     <t>capital 
 prestado</t>
@@ -118,6 +118,21 @@
   </si>
   <si>
     <t>TOTAL</t>
+  </si>
+  <si>
+    <t>parte papa</t>
+  </si>
+  <si>
+    <t>impuestos donaciones papa</t>
+  </si>
+  <si>
+    <t>ROUNDED</t>
+  </si>
+  <si>
+    <t>donacion papa liquido</t>
+  </si>
+  <si>
+    <t>donacion papa piso</t>
   </si>
 </sst>
 </file>
@@ -453,13 +468,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D5808DF-2D0F-4576-99CF-A0E928AD7DF2}">
-  <dimension ref="B2:C11"/>
+  <dimension ref="B2:L15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>15</v>
       </c>
@@ -467,23 +482,35 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B3">
         <v>58000</v>
       </c>
       <c r="C3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="K3">
+        <v>160000</v>
+      </c>
+      <c r="L3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B4">
         <v>124160</v>
       </c>
       <c r="C4" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="K4">
+        <v>128000</v>
+      </c>
+      <c r="L4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B5">
         <v>128000</v>
       </c>
@@ -491,41 +518,68 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B6">
+        <v>128000</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B7">
         <f>100000-73570</f>
         <v>26430</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C7" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B7">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B8">
         <v>-73570</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B8" s="5">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B9" s="5">
         <f>amort1_29840!E233</f>
         <v>116259.53000000062</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C9" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B10" t="s">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B10">
+        <v>1193</v>
+      </c>
+      <c r="C10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B12" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B11">
-        <f>SUM(B3:B8)</f>
-        <v>379279.53000000061</v>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B13">
+        <f>SUM(B3:B9)</f>
+        <v>507279.53000000061</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B15">
+        <f>ROUND(B13,-4)</f>
+        <v>510000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>